<commit_message>
adiciona novo processo de tradução de dados
</commit_message>
<xml_diff>
--- a/data-manipulation-scripts/sheets-cleanup/processed_sheets/ CILINDRO MESTRE 11_02.xlsx
+++ b/data-manipulation-scripts/sheets-cleanup/processed_sheets/ CILINDRO MESTRE 11_02.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,11 +432,6 @@
           <t>QUANTIDADE</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>PREÇO</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -457,11 +452,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -482,7 +472,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -503,11 +492,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>135</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -528,11 +512,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>166</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -553,11 +532,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>166</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -578,11 +552,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -595,7 +564,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CILINDRO MESTRE FREIO RSERVATORIO SMARTFOX BIZ125 2018 A 2021</t>
+          <t>CILINDRO MESTRE FREIO RESERVATORIO SMARTFOX BIZ125 2018 A 2021</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -603,7 +572,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -616,7 +584,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CILINDRO FREIO SUPERIOR TMAC BURGMAN125 2014 TM457</t>
+          <t>CILINDRO MESTRE FREIO SUPERIOR TMAC BURGMAN125 2014 TM457</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -624,7 +592,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -637,7 +604,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CILINDRO FREIO SUPERIOR TMAC FACTOR125 150 2009 A 2016</t>
+          <t>CILINDRO MESTRE FREIO SUPERIOR TMAC FACTOR125 150 2009 A 2016</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -645,7 +612,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>